<commit_message>
last change before biorxiv submission
</commit_message>
<xml_diff>
--- a/Phenotype/Tables/EPS_TableS10A_FromR.xlsx
+++ b/Phenotype/Tables/EPS_TableS10A_FromR.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -367,25 +367,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Mean Sq</t>
+          <t>Df</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>NumDF</t>
+          <t>F value</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>DenDF</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>F value</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Pr(&gt;F)</t>
         </is>
@@ -399,28 +389,18 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0.272</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>0.272</t>
-        </is>
-      </c>
-      <c r="D2">
+          <t>0.282</t>
+        </is>
+      </c>
+      <c r="C2">
         <v>1</v>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>25.302</t>
+        </is>
+      </c>
       <c r="E2" t="inlineStr">
-        <is>
-          <t>114.402</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>14.931</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
         <is>
           <t>&lt; 0.001</t>
         </is>
@@ -434,28 +414,18 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1.526</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0.763</t>
-        </is>
-      </c>
-      <c r="D3">
+          <t>0.498</t>
+        </is>
+      </c>
+      <c r="C3">
         <v>2</v>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>22.344</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
-        <is>
-          <t>225.850</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>41.878</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
         <is>
           <t>&lt; 0.001</t>
         </is>
@@ -469,28 +439,18 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0.328</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>0.328</t>
-        </is>
-      </c>
-      <c r="D4">
+          <t>0.321</t>
+        </is>
+      </c>
+      <c r="C4">
         <v>1</v>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>28.850</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
-        <is>
-          <t>112.275</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>18.000</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
         <is>
           <t>&lt; 0.001</t>
         </is>
@@ -504,100 +464,65 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0.005</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>0.005</t>
-        </is>
-      </c>
-      <c r="D5">
+          <t>0.002</t>
+        </is>
+      </c>
+      <c r="C5">
         <v>1</v>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0.210</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>114.933</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>0.288</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>0.593</t>
+          <t>0.647</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Rep</t>
+          <t>Morphology:Variety</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0.866</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>0.289</t>
-        </is>
-      </c>
-      <c r="D6">
-        <v>3</v>
+          <t>0.004</t>
+        </is>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0.166</t>
+        </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>933.323</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>15.855</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>&lt; 0.001</t>
+          <t>0.847</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Morphology:Variety</t>
+          <t>Residuals</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0.018</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>0.009</t>
-        </is>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>238.198</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>0.482</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>0.618</t>
+          <t>3.820</t>
+        </is>
+      </c>
+      <c r="C7">
+        <v>343</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>

</xml_diff>